<commit_message>
Fix utilization band: 15 tpd all scenarios, full rev-leg 0.75
Uniform max_trips_per_day=15 across thin/mid/full; restore mature
revenue_leg_factor to 0.75. Re-run full cascade, sidecar, and Drive sheets.
</commit_message>
<xml_diff>
--- a/finance/_refresh_adani-ports.xlsx
+++ b/finance/_refresh_adani-ports.xlsx
@@ -1241,7 +1241,7 @@
       </c>
       <c r="F19" s="14" t="inlineStr">
         <is>
-          <t>Cap on revenue sailings/day — MID headline duty cycle; thin=12 / full=18 bookends in _utilization_scenarios (Jaideep 2026-06-21).</t>
+          <t>Cap on revenue sailings/day — 15 across thin/mid/full scenarios (Jaideep 2026-06-21).</t>
         </is>
       </c>
     </row>
@@ -1554,7 +1554,7 @@
         <v>0.7</v>
       </c>
       <c r="C33" s="19" t="n">
-        <v>0.85</v>
+        <v>0.75</v>
       </c>
       <c r="F33" s="14" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Clarify OPEX language in transparent sheets (no value changes)
Expand Read me OPEX glossary; rename marina/insurance/charge columns and
Assumptions labels to distinguish energy, berth admin, vessel insurance, and
fast-charge berth. Update country-reference schema docs and provenance notes.
</commit_message>
<xml_diff>
--- a/finance/_refresh_adani-ports.xlsx
+++ b/finance/_refresh_adani-ports.xlsx
@@ -27,23 +27,23 @@
     <definedName name="dwell_min">'Assumptions'!$B$18</definedName>
     <definedName name="max_tpd">'Assumptions'!$B$19</definedName>
     <definedName name="crew_factor">'Assumptions'!$B$20</definedName>
-    <definedName name="ins_pct">'Assumptions'!$B$21</definedName>
-    <definedName name="charge_berth">'Assumptions'!$B$22</definedName>
-    <definedName name="mech_uptime">'Assumptions'!$B$23</definedName>
-    <definedName name="capture">'Assumptions'!$B$24</definedName>
-    <definedName name="capture_captive">'Assumptions'!$B$25</definedName>
-    <definedName name="discount">'Assumptions'!$B$26</definedName>
-    <definedName name="diesel_co2pg">'Assumptions'!$B$27</definedName>
-    <definedName name="load_thin">'Assumptions'!$B$31</definedName>
-    <definedName name="revleg_thin">'Assumptions'!$C$31</definedName>
-    <definedName name="load_mid">'Assumptions'!$B$32</definedName>
-    <definedName name="revleg_mid">'Assumptions'!$C$32</definedName>
-    <definedName name="load_full">'Assumptions'!$B$33</definedName>
-    <definedName name="revleg_full">'Assumptions'!$C$33</definedName>
-    <definedName name="band_tbl">'Assumptions'!$A$31:$C$33</definedName>
-    <definedName name="scenario">'Assumptions'!$B$35</definedName>
-    <definedName name="load_sel">'Assumptions'!$B$36</definedName>
-    <definedName name="revleg_sel">'Assumptions'!$B$37</definedName>
+    <definedName name="mech_uptime">'Assumptions'!$B$21</definedName>
+    <definedName name="capture">'Assumptions'!$B$22</definedName>
+    <definedName name="capture_captive">'Assumptions'!$B$23</definedName>
+    <definedName name="discount">'Assumptions'!$B$24</definedName>
+    <definedName name="diesel_co2pg">'Assumptions'!$B$25</definedName>
+    <definedName name="ins_pct">'Assumptions'!$B$29</definedName>
+    <definedName name="charge_berth">'Assumptions'!$B$30</definedName>
+    <definedName name="load_thin">'Assumptions'!$B$34</definedName>
+    <definedName name="revleg_thin">'Assumptions'!$C$34</definedName>
+    <definedName name="load_mid">'Assumptions'!$B$35</definedName>
+    <definedName name="revleg_mid">'Assumptions'!$C$35</definedName>
+    <definedName name="load_full">'Assumptions'!$B$36</definedName>
+    <definedName name="revleg_full">'Assumptions'!$C$36</definedName>
+    <definedName name="band_tbl">'Assumptions'!$A$34:$C$36</definedName>
+    <definedName name="scenario">'Assumptions'!$B$38</definedName>
+    <definedName name="load_sel">'Assumptions'!$B$39</definedName>
+    <definedName name="revleg_sel">'Assumptions'!$B$40</definedName>
     <definedName name="country_opex">'Country opex'!$A$4:$G$3</definedName>
     <definedName name="som_floor_fleet">'Corridor economics'!$D$8</definedName>
     <definedName name="som_floor_rev">'Corridor economics'!$E$8</definedName>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B27"/>
+  <dimension ref="B2:B36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -695,84 +695,143 @@
     <row r="14">
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>EBITDA  = REVENUE − OPEX   (energy + captain + marina/overhead + maintenance)</t>
+          <t>EBITDA  = REVENUE − OPEX</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    OPEX = energy + crew + berth/port admin + maintenance + vessel insurance + fast-charge berth</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>PAYBACK = vessel CAPEX ÷ EBITDA</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" s="2" t="inlineStr"/>
-    </row>
     <row r="17">
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>From demand pool to fleet &amp; market size</t>
-        </is>
-      </c>
+      <c r="B17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Navier serviceable rides/yr = corridor demand pool × capture rate (10% on contested corridors; ~90% on captive sole-operator transfer legs — see the per-row Capture % column)</t>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>OPEX lines (per boat, per year — no double-counting)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Vessels supported = FLOOR(Navier rides/yr ÷ pax/yr per boat);  Market rev = vessels × rev/boat. The 'Market sizing' tab rolls these up into the SOM → SAM → TAM ladder.</t>
+          <t>Energy — variable propulsion cost: kWh on revenue sailings × local $/kWh (Country opex tab). Excludes utility demand charges.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="2" t="inlineStr"/>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Crew — fully-loaded captain + relief: local captain wage × crew FTE factor (Country opex + Assumptions).</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>The scenario toggle (what we flex)</t>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Berth &amp; port admin — fixed annual berth, port fees, and local marine admin (Country opex tab). Excludes vessel H&amp;M+P&amp;I and fast-charge infrastructure.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>'Corridor economics' has a SCENARIO cell = THIN / MID / FULL. It flexes two levers: load factor (how full the boat is) and revenue-leg factor (how many legs earn full fare). MID is the headline. Change that one cell and the whole model recomputes. The right-hand Payback THIN/MID/FULL columns always show all three at once.</t>
+          <t>Maintenance — vessel annual maintenance reserve (Assumptions tab).</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="2" t="inlineStr"/>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Vessel insurance — commercial H&amp;M + P&amp;I as % of regional CAPEX (Assumptions % × Country opex CAPEX column).</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Fast-charge berth — dedicated fast-charge berth slot + utility demand charges (Assumptions default; overridable per market). Separate from per-kWh energy and berth/port admin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>From demand pool to fleet &amp; market size</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Navier serviceable rides/yr = corridor demand pool × capture rate (10% on contested corridors; ~90% on captive sole-operator transfer legs — see the per-row Capture % column)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Vessels supported = FLOOR(Navier rides/yr ÷ pax/yr per boat);  Market rev = vessels × rev/boat. The 'Market sizing' tab rolls these up into the SOM → SAM → TAM ladder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>The scenario toggle (what we flex)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>'Corridor economics' has a SCENARIO cell = THIN / MID / FULL. It flexes load factor (occupancy) and revenue-leg factor (share of legs that earn full fare). Max trips/day is fixed across all three bands (see Assumptions). MID is the headline. Change SCENARIO and the whole model recomputes. Payback THIN/MID/FULL columns always show all three at once.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>Colour &amp; provenance legend</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="6" t="inlineStr">
+    <row r="34">
+      <c r="B34" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">   Yellow = INPUTS you can change (fare, distance, demand, weather).</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" s="7" t="inlineStr">
+    <row r="35">
+      <c r="B35" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">   Green  = COMPUTED by formula.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="B27" s="2" t="inlineStr">
+    <row r="36">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">   Every fare &amp; demand figure carries a Source tier (T1 official → T5 modeled) + Confidence (high/med/low). Null beats a wrong number: no published pool → blank, not a guess.</t>
         </is>
@@ -789,7 +848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F37"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1278,11 +1337,11 @@
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>Insurance (% of capex/yr)</t>
+          <t>Mechanical uptime</t>
         </is>
       </c>
       <c r="B21" s="17" t="n">
-        <v>0.025</v>
+        <v>0.75</v>
       </c>
       <c r="C21" s="13" t="inlineStr">
         <is>
@@ -1291,7 +1350,7 @@
       </c>
       <c r="D21" s="13" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T4</t>
         </is>
       </c>
       <c r="E21" s="13" t="inlineStr">
@@ -1301,29 +1360,25 @@
       </c>
       <c r="F21" s="14" t="inlineStr">
         <is>
-          <t>H&amp;M + P&amp;I for a commercial passenger vessel ~2.5%/yr of capex; scales with regional capex overrides (Jaideep 2026-06-19).</t>
+          <t>Blade luxury aviation ~75-80% reliability uptime</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>Charging &amp; berth (additional to marina+energy)</t>
-        </is>
-      </c>
-      <c r="B22" s="15" t="n">
-        <v>18000</v>
+          <t>Navier capture rate</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="n">
+        <v>0.1</v>
       </c>
       <c r="C22" s="13" t="inlineStr">
         <is>
-          <t>USD/yr</t>
-        </is>
-      </c>
-      <c r="D22" s="13" t="inlineStr">
-        <is>
-          <t>T3</t>
-        </is>
-      </c>
+          <t>frac</t>
+        </is>
+      </c>
+      <c r="D22" s="13" t="inlineStr"/>
       <c r="E22" s="13" t="inlineStr">
         <is>
           <t>med</t>
@@ -1331,29 +1386,25 @@
       </c>
       <c r="F22" s="14" t="inlineStr">
         <is>
-          <t>Dedicated fast-charge berth + demand charges, ADDITIONAL to marina overhead and energy (Jaideep 2026-06-19). L3-overridable.</t>
+          <t>Navier wins ~10% of a CONTESTED corridor demand pool (locked). Captive sole-operator transfer legs (captive:true / luxury_charter / hospitality archetypes) carry the captive rate instead — see per-row Capture %.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
         <is>
-          <t>Mechanical uptime</t>
+          <t>Captive capture rate (A′ corridors)</t>
         </is>
       </c>
       <c r="B23" s="17" t="n">
-        <v>0.75</v>
+        <v>0.9</v>
       </c>
       <c r="C23" s="13" t="inlineStr">
         <is>
           <t>frac</t>
         </is>
       </c>
-      <c r="D23" s="13" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
+      <c r="D23" s="13" t="inlineStr"/>
       <c r="E23" s="13" t="inlineStr">
         <is>
           <t>med</t>
@@ -1361,255 +1412,303 @@
       </c>
       <c r="F23" s="14" t="inlineStr">
         <is>
-          <t>Blade luxury aviation ~75-80% reliability uptime</t>
+          <t>Sole-operator water-access-only transfer legs (captive:true or luxury_charter/hospitality archetype): Navier IS the transfer fleet — capture ~90%. Applied per-row in the Capture % column.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>Navier capture rate</t>
-        </is>
-      </c>
-      <c r="B24" s="17" t="n">
-        <v>0.1</v>
+          <t>Discount factor (vs comparable fare)</t>
+        </is>
+      </c>
+      <c r="B24" s="16" t="n">
+        <v>1</v>
       </c>
       <c r="C24" s="13" t="inlineStr">
         <is>
           <t>frac</t>
         </is>
       </c>
-      <c r="D24" s="13" t="inlineStr"/>
+      <c r="D24" s="13" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
       <c r="E24" s="13" t="inlineStr">
         <is>
-          <t>med</t>
+          <t>high</t>
         </is>
       </c>
       <c r="F24" s="14" t="inlineStr">
         <is>
-          <t>Navier wins ~10% of a CONTESTED corridor demand pool (locked). Captive sole-operator transfer legs (captive:true / luxury_charter / hospitality archetypes) carry the captive rate instead — see per-row Capture %.</t>
+          <t>Market parity — better product, not cheaper (locked).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
         <is>
-          <t>Captive capture rate (A′ corridors)</t>
-        </is>
-      </c>
-      <c r="B25" s="17" t="n">
-        <v>0.9</v>
+          <t>Diesel CO₂ per gallon</t>
+        </is>
+      </c>
+      <c r="B25" s="16" t="n">
+        <v>10.21</v>
       </c>
       <c r="C25" s="13" t="inlineStr">
         <is>
+          <t>kg/gal</t>
+        </is>
+      </c>
+      <c r="D25" s="13" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="F25" s="14" t="inlineStr">
+        <is>
+          <t>US EPA: 10.21 kg CO2 per gallon marine/diesel</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>OPEX defaults  (global fallbacks — localized energy, crew, berth admin on Country opex tab)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="E28" s="10" t="inlineStr">
+        <is>
+          <t>Conf.</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="inlineStr">
+        <is>
+          <t>Source / note</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>Vessel insurance — H&amp;M + P&amp;I (% of CAPEX/yr)</t>
+        </is>
+      </c>
+      <c r="B29" s="17" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
           <t>frac</t>
         </is>
       </c>
-      <c r="D25" s="13" t="inlineStr"/>
-      <c r="E25" s="13" t="inlineStr">
+      <c r="D29" s="13" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="E29" s="13" t="inlineStr">
         <is>
           <t>med</t>
         </is>
       </c>
-      <c r="F25" s="14" t="inlineStr">
-        <is>
-          <t>Sole-operator water-access-only transfer legs (captive:true or luxury_charter/hospitality archetype): Navier IS the transfer fleet — capture ~90%. Applied per-row in the Capture % column.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="11" t="inlineStr">
-        <is>
-          <t>Discount factor (vs comparable fare)</t>
-        </is>
-      </c>
-      <c r="B26" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="C26" s="13" t="inlineStr">
-        <is>
-          <t>frac</t>
-        </is>
-      </c>
-      <c r="D26" s="13" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="E26" s="13" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="F26" s="14" t="inlineStr">
-        <is>
-          <t>Market parity — better product, not cheaper (locked).</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="11" t="inlineStr">
-        <is>
-          <t>Diesel CO₂ per gallon</t>
-        </is>
-      </c>
-      <c r="B27" s="16" t="n">
-        <v>10.21</v>
-      </c>
-      <c r="C27" s="13" t="inlineStr">
-        <is>
-          <t>kg/gal</t>
-        </is>
-      </c>
-      <c r="D27" s="13" t="inlineStr">
-        <is>
-          <t>T1</t>
-        </is>
-      </c>
-      <c r="E27" s="13" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="F27" s="14" t="inlineStr">
-        <is>
-          <t>US EPA: 10.21 kg CO2 per gallon marine/diesel</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>Utilization scenarios  (the two levers we flex)</t>
+      <c r="F29" s="14" t="inlineStr">
+        <is>
+          <t>Commercial vessel H&amp;M + P&amp;I ~2.5%/yr of regional CAPEX. Separate from berth/port admin in Country opex (Jaideep 2026-06-19).. Multiplied by regional CAPEX (Country opex col G). Not included in berth/port admin.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="10" t="inlineStr">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>Fast-charge berth &amp; demand charges (global default)</t>
+        </is>
+      </c>
+      <c r="B30" s="15" t="n">
+        <v>18000</v>
+      </c>
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>USD/yr</t>
+        </is>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="F30" s="14" t="inlineStr">
+        <is>
+          <t>Dedicated fast-charge berth slot + utility demand charges. Excludes per-kWh propulsion energy and berth/port admin (Jaideep 2026-06-19). L3-overridable per market.. Dedicated charge berth + utility demand charges. Excludes per-kWh propulsion energy and berth/port admin. L3-overridable per market.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="9" t="inlineStr">
+        <is>
+          <t>Utilization scenarios  (load factor + revenue-leg factor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
         <is>
           <t>Scenario</t>
         </is>
       </c>
-      <c r="B30" s="10" t="inlineStr">
+      <c r="B33" s="10" t="inlineStr">
         <is>
           <t>Load factor</t>
         </is>
       </c>
-      <c r="C30" s="10" t="inlineStr">
+      <c r="C33" s="10" t="inlineStr">
         <is>
           <t>Rev-leg factor</t>
         </is>
       </c>
-      <c r="D30" s="10" t="inlineStr"/>
-      <c r="E30" s="10" t="inlineStr"/>
-      <c r="F30" s="10" t="inlineStr">
+      <c r="D33" s="10" t="inlineStr"/>
+      <c r="E33" s="10" t="inlineStr"/>
+      <c r="F33" s="10" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="18" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="18" t="inlineStr">
         <is>
           <t>THIN</t>
         </is>
       </c>
-      <c r="B31" s="19" t="n">
+      <c r="B34" s="19" t="n">
         <v>0.45</v>
       </c>
-      <c r="C31" s="19" t="n">
+      <c r="C34" s="19" t="n">
         <v>0.55</v>
       </c>
-      <c r="F31" s="14" t="inlineStr">
+      <c r="F34" s="14" t="inlineStr">
         <is>
           <t>thin/one-way/seasonal corridor — conservative floor</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="18" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="18" t="inlineStr">
         <is>
           <t>MID</t>
         </is>
       </c>
-      <c r="B32" s="19" t="n">
+      <c r="B35" s="19" t="n">
         <v>0.55</v>
       </c>
-      <c r="C32" s="19" t="n">
+      <c r="C35" s="19" t="n">
         <v>0.65</v>
       </c>
-      <c r="F32" s="14" t="inlineStr">
+      <c r="F35" s="14" t="inlineStr">
         <is>
           <t>HEADLINE — realistic busy two-way corridor</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="18" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="18" t="inlineStr">
         <is>
           <t>FULL</t>
         </is>
       </c>
-      <c r="B33" s="19" t="n">
+      <c r="B36" s="19" t="n">
         <v>0.7</v>
       </c>
-      <c r="C33" s="19" t="n">
+      <c r="C36" s="19" t="n">
         <v>0.75</v>
       </c>
-      <c r="F33" s="14" t="inlineStr">
+      <c r="F36" s="14" t="inlineStr">
         <is>
           <t>mature/dense corridor — optimistic ceiling</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="20" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="20" t="inlineStr">
         <is>
           <t>SCENARIO (toggle me)</t>
         </is>
       </c>
-      <c r="B35" s="21" t="inlineStr">
+      <c r="B38" s="21" t="inlineStr">
         <is>
           <t>MID</t>
         </is>
       </c>
-      <c r="C35" s="22" t="inlineStr">
+      <c r="C38" s="22" t="inlineStr">
         <is>
           <t>← set THIN / MID / FULL</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="11" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="11" t="inlineStr">
         <is>
           <t>Selected load factor</t>
         </is>
       </c>
-      <c r="B36" s="23">
-        <f>VLOOKUP(scenario,'Assumptions'!$A$31:$C$33,2,FALSE)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="11" t="inlineStr">
+      <c r="B39" s="23">
+        <f>VLOOKUP(scenario,'Assumptions'!$A$34:$C$36,2,FALSE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr">
         <is>
           <t>Selected rev-leg factor</t>
         </is>
       </c>
-      <c r="B37" s="23">
-        <f>VLOOKUP(scenario,'Assumptions'!$A$31:$C$33,3,FALSE)</f>
+      <c r="B40" s="23">
+        <f>VLOOKUP(scenario,'Assumptions'!$A$34:$C$36,3,FALSE)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A3:F3"/>
+  <mergeCells count="5">
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A29:F29"/>
+    <mergeCell ref="A32:F32"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A3:F3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="B35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"THIN,MID,FULL"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1639,7 +1738,7 @@
     <row r="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>Country opex — L3 localized layer (VLOOKUP target for the engine)</t>
+          <t>Country opex — localized inputs (crew, energy, berth admin, CAPEX)</t>
         </is>
       </c>
     </row>
@@ -1666,7 +1765,7 @@
       </c>
       <c r="E3" s="24" t="inlineStr">
         <is>
-          <t>Marina $/yr</t>
+          <t>Berth &amp; port admin $/yr</t>
         </is>
       </c>
       <c r="F3" s="24" t="inlineStr">
@@ -1681,7 +1780,7 @@
       </c>
       <c r="H3" s="24" t="inlineStr">
         <is>
-          <t>Source notes (captain | energy | marina)</t>
+          <t>Source notes (crew | energy | berth admin)</t>
         </is>
       </c>
     </row>
@@ -1724,10 +1823,10 @@
     <col width="11" customWidth="1" min="20" max="20"/>
     <col width="10" customWidth="1" min="21" max="21"/>
     <col width="10" customWidth="1" min="22" max="22"/>
-    <col width="10" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
     <col width="9" customWidth="1" min="24" max="24"/>
-    <col width="10" customWidth="1" min="25" max="25"/>
-    <col width="11" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="25" max="25"/>
+    <col width="12" customWidth="1" min="26" max="26"/>
     <col width="11" customWidth="1" min="27" max="27"/>
     <col width="10" customWidth="1" min="28" max="28"/>
     <col width="11" customWidth="1" min="29" max="29"/>
@@ -1888,7 +1987,7 @@
       </c>
       <c r="W3" s="24" t="inlineStr">
         <is>
-          <t>Marina/yr</t>
+          <t>Berth &amp; port admin/yr</t>
         </is>
       </c>
       <c r="X3" s="24" t="inlineStr">
@@ -1898,12 +1997,12 @@
       </c>
       <c r="Y3" s="24" t="inlineStr">
         <is>
-          <t>Insurance/yr</t>
+          <t>Vessel insurance/yr</t>
         </is>
       </c>
       <c r="Z3" s="24" t="inlineStr">
         <is>
-          <t>Charge+berth/yr</t>
+          <t>Fast-charge berth/yr</t>
         </is>
       </c>
       <c r="AA3" s="24" t="inlineStr">

</xml_diff>